<commit_message>
HeliSR Rev 4.0: 1206 resistors and caps on the back
C4 and R1-R11 go from 0805 to 1206, so every resistor and capacitor on
the board is 1206 (C4 is now the same part as C1/C2). The back parts are
re-placed for the larger size and the board is re-routed (best of 45
variants: complete, 44 router vias, no neck-downs). DRC clean at every
severity with a new rule for RST's courtyard between the far-end ports;
netlist check passes. The stitching search keeps a 0.05 mm margin over
the hole-to-hole rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PCB/HeliSR_Rev4.0/HeliSR_Rev4.0_Board_BOM.xlsx
+++ b/PCB/HeliSR_Rev4.0/HeliSR_Rev4.0_Board_BOM.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The parts you solder onto the bare HeliSR Rev 4.0 PCB, checked against the board file. Rev 4.0 has not been ordered. The front carries the connectors, the button and Rev 3.0's parts; the back carries U3, C4 and R1-R11. The Pro Micro and its pin headers are listed separately at the end. Unit prices for the parts carried over from Rev 3.0 are single-unit Digi-Key prices from the Rev 3.0 cart (2026-10-19 to 2026-10-22). The new Rev 4.0 parts are priced from distributor listings found on 2026-10-26 (PCA9546ADR: Digi-Key cut tape; BM04B-SRSS-TBT: Digi-Key via an aggregator) or, for the 0805 resistors and capacitor, at the Rev 3.0 0805 resistor's price: check them in the cart. Before shipping and tariff. The bare PCB is priced at a third of an OSH Park order of three (Rev 3.0: $10.20).</t>
+          <t>The parts you solder onto the bare HeliSR Rev 4.0 PCB, checked against the board file. Rev 4.0 has not been ordered. The front carries the connectors, the button and Rev 3.0's parts; the back carries U3, C4 and R1-R11. Every resistor and capacitor is 1206. The Pro Micro and its pin headers are listed separately at the end. Unit prices for the parts carried over from Rev 3.0 are single-unit Digi-Key prices from the Rev 3.0 cart (2026-10-19 to 2026-10-22). The new Rev 4.0 parts are priced from distributor listings found on 2026-10-26 (PCA9546ADR: Digi-Key cut tape; BM04B-SRSS-TBT: Digi-Key via an aggregator) or, for the 1206 resistors, at the Rev 3.0 0805 resistor's price: check them in the cart. Before shipping and tariff. The bare PCB is priced at a third of an OSH Park order of three (Rev 3.0: $10.20).</t>
         </is>
       </c>
     </row>
@@ -813,11 +813,11 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>C1, C2</t>
+          <t>C1, C2, C4</t>
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="10">
         <f>C9*$C$3</f>
@@ -862,7 +862,7 @@
       </c>
       <c r="M9" s="11" t="inlineStr">
         <is>
-          <t>Decoupling: C1 beside U1's VCC pin, C2 beside U2's</t>
+          <t>Decoupling: C1 beside U1's VCC pin, C2 beside U2's (front); C4 beside U3's (back)</t>
         </is>
       </c>
     </row>
@@ -990,11 +990,11 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>R1-R8</t>
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D12" s="10">
         <f>C12*$C$3</f>
@@ -1002,32 +1002,32 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>100nF</t>
+          <t>2.2k</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Capacitor, 100 nF, 50 V, X7R, 0805</t>
+          <t>Resistor, 2.2 kOhm, 1 %, 1/4 W, 1206</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>C_0805_2012Metric</t>
+          <t>R_1206_3216Metric</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>CL21B104KBCNNNC</t>
+          <t>RC1206FR-072K2L</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>1276-1003-1-ND</t>
+          <t>311-2.20KFRCT-ND</t>
         </is>
       </c>
       <c r="K12" s="13" t="n">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="M12" s="11" t="inlineStr">
         <is>
-          <t>Back, beside U3's VCC pin</t>
+          <t>Back: the ports' I2C pull-ups, a pair under each port (R1/R2 AX1, R3/R4 AX2, R5/R6 AX3, R7/R8 AX4; the odd one SDA, the even one SCL)</t>
         </is>
       </c>
     </row>
@@ -1049,11 +1049,11 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>R1-R8</t>
+          <t>R9-R11</t>
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D13" s="10">
         <f>C13*$C$3</f>
@@ -1061,17 +1061,17 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>2.2k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Resistor, 2.2 kOhm, 1 %, 1/8 W, 0805</t>
+          <t>Resistor, 10 kOhm, 1 %, 1/4 W, 1206</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>R_1206_3216Metric</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
@@ -1081,12 +1081,12 @@
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>RC0805FR-072K2L</t>
+          <t>RC1206FR-0710KL</t>
         </is>
       </c>
       <c r="J13" s="12" t="inlineStr">
         <is>
-          <t>311-2.20KCRCT-ND</t>
+          <t>311-10.0KFRCT-ND</t>
         </is>
       </c>
       <c r="K13" s="13" t="n">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="M13" s="11" t="inlineStr">
         <is>
-          <t>Back: the ports' I2C pull-ups, a pair under each port (R1/R2 AX1, R3/R4 AX2, R5/R6 AX3, R7/R8 AX4; the odd one SDA, the even one SCL)</t>
+          <t>Back: pull-ups on the Pro Micro's SDA (R9) and SCL (R10), and on U3's /RESET (R11). Any 1 % 1206 10 kOhm resistor will do if this one is out of stock</t>
         </is>
       </c>
     </row>
@@ -1108,11 +1108,11 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>R9-R11</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D14" s="10">
         <f>C14*$C$3</f>
@@ -1120,36 +1120,36 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>TL1015AF160QG</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Resistor, 10 kOhm, 1 %, 1/8 W, 0805</t>
+          <t>Tactile switch, SMD, 3.9 x 2.9 mm, gull wing</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>R_0805_2012Metric</t>
+          <t>SW_TL1015AF160QG</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>E-Switch</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>RC0805FR-0710KL</t>
+          <t>TL1015AF160QG</t>
         </is>
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>311-10.0KCRCT-ND</t>
+          <t>EG4344CT-ND</t>
         </is>
       </c>
       <c r="K14" s="13" t="n">
-        <v>0.1</v>
+        <v>0.48</v>
       </c>
       <c r="L14" s="13">
         <f>IF(K14="","",D14*K14)</f>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="M14" s="11" t="inlineStr">
         <is>
-          <t>Back: pull-ups on the Pro Micro's SDA (R9) and SCL (R10), and on U3's /RESET (R11)</t>
+          <t>RST, at the far end between AX4 and AX2. The four ground tabs are left unsoldered</t>
         </is>
       </c>
     </row>
@@ -1167,11 +1167,11 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>SW1</t>
+          <t>J1, J2</t>
         </is>
       </c>
       <c r="C15" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" s="10">
         <f>C15*$C$3</f>
@@ -1179,36 +1179,36 @@
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>TL1015AF160QG</t>
+          <t>Inputs 1-8, Inputs 9-16</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Tactile switch, SMD, 3.9 x 2.9 mm, gull wing</t>
+          <t>JST SR/SH header, 10-pin, 1.0 mm, SMD, top entry</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>SW_TL1015AF160QG</t>
+          <t>JST_SH_BM10B-SRSS-TB_1x10-1MP_P1.00mm_Vertical</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>E-Switch</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>TL1015AF160QG</t>
+          <t>BM10B-SRSS-TBT</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>EG4344CT-ND</t>
+          <t>455-BM10B-SRSS-TBTCT-ND</t>
         </is>
       </c>
       <c r="K15" s="13" t="n">
-        <v>0.48</v>
+        <v>1.19</v>
       </c>
       <c r="L15" s="13">
         <f>IF(K15="","",D15*K15)</f>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="M15" s="11" t="inlineStr">
         <is>
-          <t>RST, at the far end between AX4 and AX2. The four ground tabs are left unsoldered</t>
+          <t>Switch inputs: J1 IN1-IN8, J2 IN9-IN16. Digi-Key estimates $0.33 tariff each on top</t>
         </is>
       </c>
     </row>
@@ -1226,11 +1226,11 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>J1, J2</t>
+          <t>J11-J14</t>
         </is>
       </c>
       <c r="C16" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D16" s="10">
         <f>C16*$C$3</f>
@@ -1238,17 +1238,17 @@
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Inputs 1-8, Inputs 9-16</t>
+          <t>AX1 (I2C), AX2 (I2C), AX3 (I2C), AX4 (I2C)</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>JST SR/SH header, 10-pin, 1.0 mm, SMD, top entry</t>
+          <t>JST SR/SH header, 4-pin, 1.0 mm, SMD, top entry</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>JST_SH_BM10B-SRSS-TB_1x10-1MP_P1.00mm_Vertical</t>
+          <t>JST_SH_BM04B-SRSS-TB_1x04-1MP_P1.00mm_Vertical</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1258,16 +1258,16 @@
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>BM10B-SRSS-TBT</t>
+          <t>BM04B-SRSS-TBT</t>
         </is>
       </c>
       <c r="J16" s="12" t="inlineStr">
         <is>
-          <t>455-BM10B-SRSS-TBTCT-ND</t>
+          <t>455-BM04B-SRSS-TBTCT-ND</t>
         </is>
       </c>
       <c r="K16" s="13" t="n">
-        <v>1.19</v>
+        <v>0.71</v>
       </c>
       <c r="L16" s="13">
         <f>IF(K16="","",D16*K16)</f>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M16" s="11" t="inlineStr">
         <is>
-          <t>Switch inputs: J1 IN1-IN8, J2 IN9-IN16. Digi-Key estimates $0.33 tariff each on top</t>
+          <t>AS5600 ports AX1-AX4 (J11-J14): 1 SDA, 2 GND, 3 VCC, 4 SCL. Fit all four, or only the ports you use</t>
         </is>
       </c>
     </row>
@@ -1285,11 +1285,11 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>J11-J14</t>
+          <t>J7, J8</t>
         </is>
       </c>
       <c r="C17" s="10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D17" s="10">
         <f>C17*$C$3</f>
@@ -1297,36 +1297,36 @@
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>AX1 (I2C), AX2 (I2C), AX3 (I2C), AX4 (I2C)</t>
+          <t>Pro Micro pins 1-12, Pro Micro pins 13-24</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>JST SR/SH header, 4-pin, 1.0 mm, SMD, top entry</t>
+          <t>Socket header, female, 1x12, 2.54 mm, through hole</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>JST_SH_BM04B-SRSS-TB_1x04-1MP_P1.00mm_Vertical</t>
+          <t>PinSocket_1x12_P2.54mm_Vertical</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Sullins</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>BM04B-SRSS-TBT</t>
+          <t>PPTC121LFBN-RC</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
-          <t>455-BM04B-SRSS-TBTCT-ND</t>
+          <t>S6100-ND</t>
         </is>
       </c>
       <c r="K17" s="13" t="n">
-        <v>0.71</v>
+        <v>0.75</v>
       </c>
       <c r="L17" s="13">
         <f>IF(K17="","",D17*K17)</f>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="M17" s="11" t="inlineStr">
         <is>
-          <t>AS5600 ports AX1-AX4 (J11-J14): 1 SDA, 2 GND, 3 VCC, 4 SCL. Fit all four, or only the ports you use</t>
+          <t>Pro Micro sockets. Fit last</t>
         </is>
       </c>
     </row>
@@ -1344,11 +1344,11 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>J7, J8</t>
+          <t>PCB</t>
         </is>
       </c>
       <c r="C18" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="10">
         <f>C18*$C$3</f>
@@ -1356,36 +1356,24 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Pro Micro pins 1-12, Pro Micro pins 13-24</t>
+          <t>HeliSR Rev 4.0</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>Socket header, female, 1x12, 2.54 mm, through hole</t>
-        </is>
-      </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>PinSocket_1x12_P2.54mm_Vertical</t>
-        </is>
-      </c>
+          <t>Bare PCB (no parts fitted), 2 layers, 1.6 mm FR4, 39.3 x 33.64 mm</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr"/>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>Sullins</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t>PPTC121LFBN-RC</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="inlineStr">
-        <is>
-          <t>S6100-ND</t>
-        </is>
-      </c>
+          <t>OSH Park</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr"/>
+      <c r="J18" s="11" t="inlineStr"/>
       <c r="K18" s="13" t="n">
-        <v>0.75</v>
+        <v>3.4</v>
       </c>
       <c r="L18" s="13">
         <f>IF(K18="","",D18*K18)</f>
@@ -1393,86 +1381,90 @@
       </c>
       <c r="M18" s="11" t="inlineStr">
         <is>
-          <t>Pro Micro sockets. Fit last</t>
+          <t>Not ordered yet. Priced as Rev 3.0: $10.20 for three bare boards from OSH Park</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n">
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="L19" s="14">
+        <f>SUM(L7:L18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Plugs into the board (the Pro Micro and its headers)</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8" t="n"/>
+      <c r="K20" s="8" t="n"/>
+      <c r="L20" s="8" t="n"/>
+      <c r="M20" s="9" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>PCB</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="n">
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="10">
-        <f>C19*$C$3</f>
-        <v/>
-      </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>HeliSR Rev 4.0</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>Bare PCB (no parts fitted), 2 layers, 1.6 mm FR4, 39.3 x 33.64 mm</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr"/>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>OSH Park</t>
-        </is>
-      </c>
-      <c r="I19" s="11" t="inlineStr"/>
-      <c r="J19" s="11" t="inlineStr"/>
-      <c r="K19" s="13" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="L19" s="13">
-        <f>IF(K19="","",D19*K19)</f>
-        <v/>
-      </c>
-      <c r="M19" s="11" t="inlineStr">
-        <is>
-          <t>Not ordered yet. Priced as Rev 3.0: $10.20 for three bare boards from OSH Park</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="L20" s="14">
-        <f>SUM(L7:L19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Plugs into the board (the Pro Micro and its headers)</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
-      <c r="H21" s="8" t="n"/>
-      <c r="I21" s="8" t="n"/>
-      <c r="J21" s="8" t="n"/>
-      <c r="K21" s="8" t="n"/>
-      <c r="L21" s="8" t="n"/>
-      <c r="M21" s="9" t="n"/>
+      <c r="D21" s="10">
+        <f>C21*$C$3</f>
+        <v/>
+      </c>
+      <c r="E21" s="11" t="inlineStr"/>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Pro Micro 5V/16 MHz, ATmega32U4</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr"/>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>SparkFun</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>12640</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="inlineStr">
+        <is>
+          <t>1568-12640-ND</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="n">
+        <v>23.99</v>
+      </c>
+      <c r="L21" s="13">
+        <f>IF(K21="","",D21*K21)</f>
+        <v/>
+      </c>
+      <c r="M21" s="11" t="inlineStr">
+        <is>
+          <t>Runs the HeliSR firmware (Rev 4.0 build). Plugs into J7/J8</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n">
@@ -1484,7 +1476,7 @@
         </is>
       </c>
       <c r="C22" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="10">
         <f>C22*$C$3</f>
@@ -1493,27 +1485,27 @@
       <c r="E22" s="11" t="inlineStr"/>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>Pro Micro 5V/16 MHz, ATmega32U4</t>
+          <t>Pin header, male, 1x12, 2.54 mm</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr"/>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>SparkFun</t>
+          <t>Sullins</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>12640</t>
+          <t>PRPC012SAAN-RC</t>
         </is>
       </c>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>1568-12640-ND</t>
+          <t>35-PRPC012SAAN-RC-ND</t>
         </is>
       </c>
       <c r="K22" s="13" t="n">
-        <v>23.99</v>
+        <v>0.24</v>
       </c>
       <c r="L22" s="13">
         <f>IF(K22="","",D22*K22)</f>
@@ -1521,85 +1513,34 @@
       </c>
       <c r="M22" s="11" t="inlineStr">
         <is>
-          <t>Runs the HeliSR firmware (Rev 4.0 build). Plugs into J7/J8</t>
+          <t>Soldered to the Pro Micro</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Module</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D23" s="10">
-        <f>C23*$C$3</f>
-        <v/>
-      </c>
-      <c r="E23" s="11" t="inlineStr"/>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Pin header, male, 1x12, 2.54 mm</t>
-        </is>
-      </c>
-      <c r="G23" s="11" t="inlineStr"/>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>Sullins</t>
-        </is>
-      </c>
-      <c r="I23" s="11" t="inlineStr">
-        <is>
-          <t>PRPC012SAAN-RC</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="inlineStr">
-        <is>
-          <t>35-PRPC012SAAN-RC-ND</t>
-        </is>
-      </c>
-      <c r="K23" s="13" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="L23" s="13">
-        <f>IF(K23="","",D23*K23)</f>
-        <v/>
-      </c>
-      <c r="M23" s="11" t="inlineStr">
-        <is>
-          <t>Soldered to the Pro Micro</t>
-        </is>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="L23" s="14">
+        <f>SUM(L21:L22)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="L24" s="14">
-        <f>SUM(L22:L23)</f>
+        <f>L19+L23</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="L25" s="14">
-        <f>L20+L24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>The bare PCB counts as a third of an OSH Park order of three ($10.20 for Rev 3.0).</t>
         </is>
@@ -1609,9 +1550,9 @@
   <mergeCells count="6">
     <mergeCell ref="A6:M6"/>
     <mergeCell ref="D3:M3"/>
-    <mergeCell ref="A26:M26"/>
-    <mergeCell ref="A21:M21"/>
     <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A25:M25"/>
+    <mergeCell ref="A20:M20"/>
     <mergeCell ref="A3:B3"/>
   </mergeCells>
   <hyperlinks>
@@ -1626,9 +1567,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>